<commit_message>
Add variable description table
</commit_message>
<xml_diff>
--- a/Supplementary_Table_S1_Data_Dictionary_v1.0.xlsx
+++ b/Supplementary_Table_S1_Data_Dictionary_v1.0.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12255" activeTab="1"/>
+    <workbookView windowWidth="22188" windowHeight="9060"/>
   </bookViews>
   <sheets>
     <sheet name="Supplementary Table S1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="378">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="380">
   <si>
     <t>Supplementary Table S1. Data dictionary for the seasonal-frozen-ground strong-motion flatfile</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>4.0 ≤ M</t>
     </r>
     <r>
@@ -528,6 +534,12 @@
   </si>
   <si>
     <t>m</t>
+  </si>
+  <si>
+    <t>GEBCO_2025 Grid</t>
+  </si>
+  <si>
+    <t>Nearest-grid-cell elevation extracted from the GEBCO_2025 Grid using the station coordinates.</t>
   </si>
   <si>
     <t>Metres above sea level</t>
@@ -1721,6 +1733,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F2937"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
       <t>R</t>
     </r>
     <r>
@@ -3173,7 +3191,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K100"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
@@ -3860,13 +3878,13 @@
         <v>37</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>92</v>
+        <v>117</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="J23" s="23" t="s">
         <v>18</v>
@@ -3878,178 +3896,178 @@
     <row r="24" ht="24" customHeight="1" spans="1:11">
       <c r="A24" s="25"/>
       <c r="B24" s="20" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F24" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H24" s="21" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I24" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J24" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K24" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:11">
       <c r="A25" s="25"/>
       <c r="B25" s="22" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F25" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H25" s="23" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I25" s="23" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="J25" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K25" s="23" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1" spans="1:11">
       <c r="A26" s="25"/>
       <c r="B26" s="20" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C26" s="20" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E26" s="21" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F26" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H26" s="21" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="I26" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J26" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K26" s="21" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1" spans="1:11">
       <c r="A27" s="25"/>
       <c r="B27" s="22" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H27" s="23" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I27" s="23" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="J27" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K27" s="23" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1" spans="1:11">
       <c r="A28" s="25"/>
       <c r="B28" s="20" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C28" s="20" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F28" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H28" s="21" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I28" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J28" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K28" s="21" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1" spans="1:11">
       <c r="A29" s="25"/>
       <c r="B29" s="22" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E29" s="23" t="s">
         <v>46</v>
@@ -4058,46 +4076,46 @@
         <v>37</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H29" s="23" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I29" s="23" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J29" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K29" s="23" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1" spans="1:11">
       <c r="A30" s="25"/>
       <c r="B30" s="20" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F30" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G30" s="21" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H30" s="21" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I30" s="21" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="J30" s="21" t="s">
         <v>18</v>
@@ -4109,13 +4127,13 @@
     <row r="31" ht="24" customHeight="1" spans="1:11">
       <c r="A31" s="26"/>
       <c r="B31" s="22" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E31" s="23" t="s">
         <v>52</v>
@@ -4124,33 +4142,33 @@
         <v>19</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H31" s="23" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="I31" s="23" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J31" s="23">
         <v>-999</v>
       </c>
       <c r="K31" s="23" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1" spans="1:11">
       <c r="A32" s="27" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E32" s="21" t="s">
         <v>46</v>
@@ -4159,13 +4177,13 @@
         <v>37</v>
       </c>
       <c r="G32" s="21" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H32" s="21" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I32" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J32" s="21" t="s">
         <v>18</v>
@@ -4177,13 +4195,13 @@
     <row r="33" ht="24" customHeight="1" spans="1:11">
       <c r="A33" s="28"/>
       <c r="B33" s="22" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E33" s="23" t="s">
         <v>46</v>
@@ -4192,31 +4210,31 @@
         <v>37</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H33" s="23" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="I33" s="23" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J33" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K33" s="23" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="34" ht="72" customHeight="1" spans="1:11">
       <c r="A34" s="29"/>
       <c r="B34" s="20" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C34" s="20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D34" s="21" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E34" s="21" t="s">
         <v>46</v>
@@ -4225,914 +4243,914 @@
         <v>37</v>
       </c>
       <c r="G34" s="21" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H34" s="21" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I34" s="21" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J34" s="21">
         <v>-999</v>
       </c>
       <c r="K34" s="21" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" ht="24" customHeight="1" spans="1:11">
       <c r="A35" s="30" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B35" s="22" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F35" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H35" s="23" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I35" s="23" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J35" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K35" s="23" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="36" ht="24" customHeight="1" spans="1:11">
       <c r="A36" s="31"/>
       <c r="B36" s="20" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C36" s="20" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F36" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G36" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H36" s="21" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I36" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J36" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K36" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" ht="24" customHeight="1" spans="1:11">
       <c r="A37" s="31"/>
       <c r="B37" s="22" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F37" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H37" s="23" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I37" s="23" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J37" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K37" s="23" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="38" ht="24" customHeight="1" spans="1:11">
       <c r="A38" s="31"/>
       <c r="B38" s="20" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C38" s="20" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F38" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G38" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H38" s="21" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I38" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J38" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K38" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" ht="24" customHeight="1" spans="1:11">
       <c r="A39" s="31"/>
       <c r="B39" s="22" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F39" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H39" s="23" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I39" s="23" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J39" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K39" s="23" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" ht="24" customHeight="1" spans="1:11">
       <c r="A40" s="32"/>
       <c r="B40" s="20" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C40" s="20" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D40" s="21" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F40" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G40" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H40" s="21" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I40" s="21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J40" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K40" s="21" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" ht="24" customHeight="1" spans="1:11">
       <c r="A41" s="33" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B41" s="22" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F41" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H41" s="23" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="I41" s="23" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J41" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K41" s="23" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="42" ht="36" customHeight="1" spans="1:11">
       <c r="A42" s="34"/>
       <c r="B42" s="20" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C42" s="20" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D42" s="21" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E42" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F42" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G42" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H42" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I42" s="21" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="J42" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K42" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43" ht="36" customHeight="1" spans="1:11">
       <c r="A43" s="34"/>
       <c r="B43" s="22" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F43" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H43" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I43" s="23" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J43" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K43" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" ht="36" customHeight="1" spans="1:11">
       <c r="A44" s="34"/>
       <c r="B44" s="20" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C44" s="20" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D44" s="21" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="E44" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F44" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G44" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H44" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I44" s="21" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="J44" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K44" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="45" ht="36" customHeight="1" spans="1:11">
       <c r="A45" s="34"/>
       <c r="B45" s="22" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F45" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H45" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I45" s="23" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="J45" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K45" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="46" ht="36" customHeight="1" spans="1:11">
       <c r="A46" s="34"/>
       <c r="B46" s="20" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C46" s="20" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D46" s="21" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E46" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F46" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G46" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H46" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I46" s="21" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="J46" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K46" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="47" ht="36" customHeight="1" spans="1:11">
       <c r="A47" s="34"/>
       <c r="B47" s="22" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F47" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H47" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I47" s="23" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="J47" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K47" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="48" ht="36" customHeight="1" spans="1:11">
       <c r="A48" s="34"/>
       <c r="B48" s="20" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C48" s="20" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D48" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E48" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F48" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G48" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H48" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I48" s="21" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="J48" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K48" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="49" ht="36" customHeight="1" spans="1:11">
       <c r="A49" s="34"/>
       <c r="B49" s="22" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F49" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H49" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I49" s="23" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="J49" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K49" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="50" ht="36" customHeight="1" spans="1:11">
       <c r="A50" s="34"/>
       <c r="B50" s="20" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C50" s="20" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D50" s="21" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F50" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G50" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H50" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I50" s="21" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="J50" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K50" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="51" ht="36" customHeight="1" spans="1:11">
       <c r="A51" s="34"/>
       <c r="B51" s="22" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F51" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H51" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I51" s="23" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="J51" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K51" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="52" ht="36" customHeight="1" spans="1:11">
       <c r="A52" s="34"/>
       <c r="B52" s="20" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C52" s="20" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D52" s="21" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F52" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G52" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H52" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I52" s="21" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="J52" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K52" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="53" ht="36" customHeight="1" spans="1:11">
       <c r="A53" s="34"/>
       <c r="B53" s="22" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E53" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F53" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G53" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H53" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I53" s="23" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="J53" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K53" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="54" ht="36" customHeight="1" spans="1:11">
       <c r="A54" s="34"/>
       <c r="B54" s="20" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C54" s="20" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D54" s="21" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E54" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F54" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G54" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H54" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I54" s="21" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="J54" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K54" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="55" ht="36" customHeight="1" spans="1:11">
       <c r="A55" s="34"/>
       <c r="B55" s="22" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="E55" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F55" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G55" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H55" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I55" s="23" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="J55" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K55" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="56" ht="36" customHeight="1" spans="1:11">
       <c r="A56" s="34"/>
       <c r="B56" s="20" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C56" s="20" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D56" s="21" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F56" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H56" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I56" s="21" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="J56" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K56" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="57" ht="36" customHeight="1" spans="1:11">
       <c r="A57" s="34"/>
       <c r="B57" s="22" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="E57" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F57" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G57" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H57" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I57" s="23" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="J57" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K57" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="58" ht="36" customHeight="1" spans="1:11">
       <c r="A58" s="34"/>
       <c r="B58" s="20" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C58" s="20" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D58" s="21" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="E58" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F58" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H58" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I58" s="21" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J58" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K58" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="59" ht="36" customHeight="1" spans="1:11">
       <c r="A59" s="34"/>
       <c r="B59" s="22" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E59" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F59" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G59" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H59" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I59" s="23" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J59" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K59" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" ht="36" customHeight="1" spans="1:11">
       <c r="A60" s="34"/>
       <c r="B60" s="20" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C60" s="20" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D60" s="21" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E60" s="21" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F60" s="21" t="s">
         <v>37</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H60" s="21" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I60" s="21" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="J60" s="21" t="s">
         <v>18</v>
       </c>
       <c r="K60" s="21" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="61" ht="36" customHeight="1" spans="1:11">
       <c r="A61" s="35"/>
       <c r="B61" s="22" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E61" s="23" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F61" s="23" t="s">
         <v>37</v>
       </c>
       <c r="G61" s="23" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H61" s="23" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I61" s="23" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="J61" s="23" t="s">
         <v>18</v>
       </c>
       <c r="K61" s="23" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -5662,7 +5680,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K100"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="27" style="1" customWidth="1"/>
     <col min="2" max="2" width="22" style="1" customWidth="1"/>
@@ -5674,7 +5692,7 @@
   <sheetData>
     <row r="1" ht="16.8" customHeight="1" spans="1:11">
       <c r="A1" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5702,19 +5720,19 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:11">
       <c r="A3" s="4" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -5728,16 +5746,16 @@
         <v>50</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -5751,16 +5769,16 @@
         <v>50</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>318</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>316</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>317</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>314</v>
-      </c>
       <c r="E5" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -5774,16 +5792,16 @@
         <v>50</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -5797,16 +5815,16 @@
         <v>50</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -5823,13 +5841,13 @@
         <v>56</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -5843,16 +5861,16 @@
         <v>59</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -5869,13 +5887,13 @@
         <v>97</v>
       </c>
       <c r="C10" s="8" t="s">
+        <v>331</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>329</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>327</v>
-      </c>
       <c r="E10" s="9" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -5892,13 +5910,13 @@
         <v>113</v>
       </c>
       <c r="C11" s="8" t="s">
+        <v>332</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>329</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>330</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>328</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -5912,16 +5930,16 @@
         <v>66</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -5935,16 +5953,16 @@
         <v>66</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>337</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>338</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>335</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="E13" s="9" t="s">
         <v>336</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>333</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>334</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -5958,16 +5976,16 @@
         <v>66</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -5984,13 +6002,13 @@
         <v>56</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -6001,19 +6019,19 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:11">
       <c r="A16" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B16" s="8">
         <v>0</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -6024,19 +6042,19 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:11">
       <c r="A17" s="7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B17" s="8">
         <v>1</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -6047,19 +6065,19 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:11">
       <c r="A18" s="7" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -6070,19 +6088,19 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:11">
       <c r="A19" s="7" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B19" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="E19" s="9" t="s">
         <v>349</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>346</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>347</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -6093,19 +6111,19 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:11">
       <c r="A20" s="7" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -6116,19 +6134,19 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:11">
       <c r="A21" s="7" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -6139,19 +6157,19 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:11">
       <c r="A22" s="7" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -6188,7 +6206,7 @@
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:11">
       <c r="A25" s="11" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -6216,19 +6234,19 @@
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:11">
       <c r="A27" s="4" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -6242,16 +6260,16 @@
         <v>1</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D28" s="8" t="s">
         <v>59</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -6265,16 +6283,16 @@
         <v>2</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>50</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -6288,16 +6306,16 @@
         <v>3</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -6311,16 +6329,16 @@
         <v>4</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -6334,16 +6352,16 @@
         <v>5</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>

</xml_diff>